<commit_message>
upload BUG REPORT 2
</commit_message>
<xml_diff>
--- a/documentation/BUG REPORT.xlsx
+++ b/documentation/BUG REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CDC12F-BB8D-4A2A-900C-CA4DB03964EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD3DFA0-5728-4B77-8F28-F5ACC32D3FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{99208258-F126-4562-88E1-3DA1320E1714}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>Module</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>Registration Module</t>
+  </si>
+  <si>
+    <t>Login Module</t>
   </si>
   <si>
     <t>BUG ID</t>
@@ -86,6 +89,25 @@
   </si>
   <si>
     <t>Syaif</t>
+  </si>
+  <si>
+    <t>Verify error when email not registered</t>
+  </si>
+  <si>
+    <t>BUG-02</t>
+  </si>
+  <si>
+    <t>System appears invalid email but the message not "Email and passwordincorrect" 
+(Must changed)</t>
+  </si>
+  <si>
+    <t>1. Enter unregistered email 
+2. Enter any password 
+3. Click Login</t>
+  </si>
+  <si>
+    <t>Chrome v145 /
+Windows 12</t>
   </si>
 </sst>
 </file>
@@ -516,39 +538,39 @@
   <sheetData>
     <row r="3" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="3:12" ht="47.25" x14ac:dyDescent="0.25">
       <c r="C4" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>2</v>
@@ -557,38 +579,58 @@
         <v>3</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="3:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="L4" s="5" t="s">
+      <c r="G5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
+      <c r="L5" s="5" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C6" s="5"/>

</xml_diff>